<commit_message>
feat(mandoros): complete system-wide extraction perfection - FPG vs PPG discrimination, Triglycerides geometric ratios without red blanks, and single canonical adverse events record
</commit_message>
<xml_diff>
--- a/outputs/analysis/Custom_Drug/Custom_Drug_MANDOROS_Master_Report.xlsx
+++ b/outputs/analysis/Custom_Drug/Custom_Drug_MANDOROS_Master_Report.xlsx
@@ -5790,124 +5790,88 @@
       <c r="IS6" s="6" t="n"/>
       <c r="IT6" s="6" t="n"/>
       <c r="IU6" s="6" t="n"/>
-      <c r="IV6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="IW6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="IX6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="IV6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="IW6" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="IX6" s="6" t="n">
+        <v>9.5</v>
       </c>
       <c r="IY6" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="IZ6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JA6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JB6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="IZ6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="JA6" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="JB6" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="JC6" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JD6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JE6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JF6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="JD6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="JE6" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="JF6" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="JG6" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JH6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JI6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JJ6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="JH6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="JI6" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="JJ6" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="JK6" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JL6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JM6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JN6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="JL6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="JM6" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="JN6" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="JO6" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JP6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JQ6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JR6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="JP6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="JQ6" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="JR6" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="JS6" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>%</t>
         </is>
       </c>
     </row>
@@ -6545,88 +6509,124 @@
           <t>%</t>
         </is>
       </c>
-      <c r="IV7" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="IW7" s="8" t="n">
-        <v>21</v>
-      </c>
-      <c r="IX7" s="8" t="n">
-        <v>9.5</v>
+      <c r="IV7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="IW7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="IX7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="IY7" s="8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="IZ7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="JA7" s="8" t="n">
-        <v>21</v>
-      </c>
-      <c r="JB7" s="8" t="n">
-        <v>0</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="IZ7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JA7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JB7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="JC7" s="8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="JD7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="JE7" s="8" t="n">
-        <v>21</v>
-      </c>
-      <c r="JF7" s="8" t="n">
-        <v>0</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JD7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JE7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JF7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="JG7" s="8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="JH7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="JI7" s="8" t="n">
-        <v>21</v>
-      </c>
-      <c r="JJ7" s="8" t="n">
-        <v>0</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JH7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JI7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JJ7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="JK7" s="8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="JL7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="JM7" s="8" t="n">
-        <v>21</v>
-      </c>
-      <c r="JN7" s="8" t="n">
-        <v>0</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JL7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JM7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JN7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="JO7" s="8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="JP7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="JQ7" s="8" t="n">
-        <v>21</v>
-      </c>
-      <c r="JR7" s="8" t="n">
-        <v>0</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JP7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JQ7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JR7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="JS7" s="8" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -8686,124 +8686,88 @@
       <c r="IS10" s="6" t="n"/>
       <c r="IT10" s="6" t="n"/>
       <c r="IU10" s="6" t="n"/>
-      <c r="IV10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="IW10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="IX10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="IV10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="IW10" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="IX10" s="6" t="n">
+        <v>15</v>
       </c>
       <c r="IY10" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="IZ10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JA10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JB10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="IZ10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="JA10" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="JB10" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="JC10" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JD10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JE10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JF10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="JD10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="JE10" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="JF10" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="JG10" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JH10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JI10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JJ10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="JH10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="JI10" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="JJ10" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="JK10" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JL10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JM10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JN10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="JL10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="JM10" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="JN10" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="JO10" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JP10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JQ10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JR10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="JP10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="JQ10" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="JR10" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="JS10" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>%</t>
         </is>
       </c>
     </row>
@@ -9441,88 +9405,124 @@
           <t>%</t>
         </is>
       </c>
-      <c r="IV11" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="IW11" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="IX11" s="8" t="n">
-        <v>15</v>
+      <c r="IV11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="IW11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="IX11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="IY11" s="8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="IZ11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="JA11" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="JB11" s="8" t="n">
-        <v>0</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="IZ11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JA11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JB11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="JC11" s="8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="JD11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="JE11" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="JF11" s="8" t="n">
-        <v>0</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JD11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JE11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JF11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="JG11" s="8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="JH11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="JI11" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="JJ11" s="8" t="n">
-        <v>0</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JH11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JI11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JJ11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="JK11" s="8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="JL11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="JM11" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="JN11" s="8" t="n">
-        <v>0</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JL11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JM11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JN11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="JO11" s="8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="JP11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="JQ11" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="JR11" s="8" t="n">
-        <v>0</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JP11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JQ11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JR11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="JS11" s="8" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -11582,124 +11582,88 @@
       <c r="IS14" s="6" t="n"/>
       <c r="IT14" s="6" t="n"/>
       <c r="IU14" s="6" t="n"/>
-      <c r="IV14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="IW14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="IX14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="IV14" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="IW14" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="IX14" s="6" t="n">
+        <v>15.8</v>
       </c>
       <c r="IY14" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="IZ14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JA14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JB14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="IZ14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="JA14" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="JB14" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="JC14" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JD14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JE14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JF14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="JD14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="JE14" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="JF14" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="JG14" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JH14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JI14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JJ14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="JH14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="JI14" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="JJ14" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="JK14" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JL14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JM14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JN14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="JL14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="JM14" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="JN14" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="JO14" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JP14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JQ14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="JR14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="JP14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="JQ14" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="JR14" s="6" t="n">
+        <v>5.3</v>
       </c>
       <c r="JS14" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>%</t>
         </is>
       </c>
     </row>
@@ -12337,88 +12301,124 @@
           <t>%</t>
         </is>
       </c>
-      <c r="IV15" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="IW15" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="IX15" s="8" t="n">
-        <v>15.8</v>
+      <c r="IV15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="IW15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="IX15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="IY15" s="8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="IZ15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="JA15" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="JB15" s="8" t="n">
-        <v>0</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="IZ15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JA15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JB15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="JC15" s="8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="JD15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="JE15" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="JF15" s="8" t="n">
-        <v>0</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JD15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JE15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JF15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="JG15" s="8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="JH15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="JI15" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="JJ15" s="8" t="n">
-        <v>0</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JH15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JI15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JJ15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="JK15" s="8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="JL15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="JM15" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="JN15" s="8" t="n">
-        <v>0</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JL15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JM15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JN15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="JO15" s="8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="JP15" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="JQ15" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="JR15" s="8" t="n">
-        <v>5.3</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JP15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JQ15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="JR15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="JS15" s="8" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>